<commit_message>
add xiaoyu and reina calcs
</commit_message>
<xml_diff>
--- a/data/azucena/output/azucena_gto.xlsx
+++ b/data/azucena/output/azucena_gto.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dfa238\pyproj\gambit_tekken8\data\azucena\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38992B06-3D11-47BB-9F1A-245C2DD65FA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8CAF0AD-EDCA-45B9-8AFF-897158356F1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12900" yWindow="2700" windowWidth="15900" windowHeight="11925" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20775" yWindow="2280" windowWidth="19320" windowHeight="11925" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Azucena Heat Engager (+17)" sheetId="1" r:id="rId1"/>
@@ -1354,7 +1354,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
-    <col min="2" max="2" width="90" customWidth="1"/>
+    <col min="2" max="2" width="77.85546875" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
   </cols>
@@ -1780,7 +1780,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.42578125" customWidth="1"/>
-    <col min="2" max="2" width="107.85546875" customWidth="1"/>
+    <col min="2" max="2" width="67.5703125" customWidth="1"/>
     <col min="3" max="3" width="21" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
   </cols>

</xml_diff>